<commit_message>
Add chained material load workflows
</commit_message>
<xml_diff>
--- a/src/centric_api/templates/style-bom-load-template.xlsx
+++ b/src/centric_api/templates/style-bom-load-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="style-bom-load" sheetId="1" r:id="Rc4bd4fcb1caa45d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="style-bom-load" sheetId="1" r:id="R7ca36da8230542d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2584,7 +2584,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d71abe1d8b54245"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R995f0a82228c4e14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>